<commit_message>
go back button in forms
</commit_message>
<xml_diff>
--- a/appraisal.xlsx
+++ b/appraisal.xlsx
@@ -520,12 +520,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>98</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>67</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -535,31 +535,31 @@
         <v>2</v>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K2" t="n">
         <v>2</v>
       </c>
       <c r="L2" t="n">
+        <v>3</v>
+      </c>
+      <c r="M2" t="n">
         <v>2</v>
       </c>
-      <c r="M2" t="n">
-        <v>1</v>
-      </c>
       <c r="N2" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="O2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>